<commit_message>
Add 12-16t excavator benchmark dashboards
</commit_message>
<xml_diff>
--- a/data/source-excel/XCMG_8-10t_mini_excavator_competitor_source.xlsx
+++ b/data/source-excel/XCMG_8-10t_mini_excavator_competitor_source.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\竞争力评价\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC62AD3A-9F1C-4243-9D33-AF1D5C7ACBA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0CC4B43-F9AE-4230-8BD1-55B297DCF8FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{B5661643-CBB0-49A1-B1C9-E50A60AA7B99}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{B5661643-CBB0-49A1-B1C9-E50A60AA7B99}"/>
   </bookViews>
   <sheets>
     <sheet name="参数" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="153">
   <si>
     <t>运输参数</t>
   </si>
@@ -323,115 +323,16 @@
     <t>三泵</t>
   </si>
   <si>
-    <t>2.6/4.7</t>
-  </si>
-  <si>
-    <t>75/55</t>
-  </si>
-  <si>
-    <t>2.6/4.4</t>
-  </si>
-  <si>
     <t>无，楔式快换</t>
   </si>
   <si>
     <t>选配2D</t>
   </si>
   <si>
-    <t>5600/5700</t>
-  </si>
-  <si>
     <t>2.8/4.6</t>
   </si>
   <si>
-    <t>70/53</t>
-  </si>
-  <si>
-    <t>2.8/5</t>
-  </si>
-  <si>
-    <t>27.3-32.2</t>
-  </si>
-  <si>
-    <t>72/50</t>
-  </si>
-  <si>
-    <t>4996-5754</t>
-  </si>
-  <si>
-    <t>4790-5557</t>
-  </si>
-  <si>
     <t>2.5/4.2</t>
-  </si>
-  <si>
-    <t>26.9-29.5</t>
-  </si>
-  <si>
-    <t>80/60</t>
-  </si>
-  <si>
-    <t>5151/5386</t>
-  </si>
-  <si>
-    <t>2.8/4.5</t>
-  </si>
-  <si>
-    <t>70/50</t>
-  </si>
-  <si>
-    <t>5555-5995</t>
-  </si>
-  <si>
-    <t>2x56.1+37</t>
-  </si>
-  <si>
-    <t>2.8/4.8</t>
-  </si>
-  <si>
-    <t>31.7-33.1</t>
-  </si>
-  <si>
-    <t>5600-6050</t>
-  </si>
-  <si>
-    <t>2x56.1+38</t>
-  </si>
-  <si>
-    <t>2.8/4.9</t>
-  </si>
-  <si>
-    <t>31.7-33.8</t>
-  </si>
-  <si>
-    <t>70/55</t>
-  </si>
-  <si>
-    <t>4940-5697</t>
-  </si>
-  <si>
-    <t>2.7/4.4</t>
-  </si>
-  <si>
-    <t>60/53</t>
-  </si>
-  <si>
-    <t>1095/1200
-（副配重）</t>
-  </si>
-  <si>
-    <t>1000/1100
-（副配重）</t>
-  </si>
-  <si>
-    <t>951/1032
-（副配重）</t>
-  </si>
-  <si>
-    <t>Closed 负载敏感</t>
-  </si>
-  <si>
-    <t>闭式 负载敏感</t>
   </si>
   <si>
     <t>工作灯延迟关闭</t>
@@ -527,6 +428,94 @@
   </si>
   <si>
     <t>标配2051mm</t>
+  </si>
+  <si>
+    <t>9250/9500</t>
+  </si>
+  <si>
+    <t>2.7/4.9</t>
+  </si>
+  <si>
+    <t>62/50</t>
+  </si>
+  <si>
+    <t>8440-9355</t>
+  </si>
+  <si>
+    <t>3.1/5.1</t>
+  </si>
+  <si>
+    <t>36.9-40.9</t>
+  </si>
+  <si>
+    <t>60/50</t>
+  </si>
+  <si>
+    <t>8726-9260</t>
+  </si>
+  <si>
+    <t>2x72+56</t>
+  </si>
+  <si>
+    <t>3.1/5</t>
+  </si>
+  <si>
+    <t>30/39</t>
+  </si>
+  <si>
+    <t>65/55</t>
+  </si>
+  <si>
+    <t>8400-8900</t>
+  </si>
+  <si>
+    <t>2x84.6</t>
+  </si>
+  <si>
+    <t>2.7/4.8</t>
+  </si>
+  <si>
+    <t>36.5-38.6</t>
+  </si>
+  <si>
+    <t>67/60</t>
+  </si>
+  <si>
+    <t>8600-10000</t>
+  </si>
+  <si>
+    <t>2x68+54</t>
+  </si>
+  <si>
+    <t>2.6/5.2</t>
+  </si>
+  <si>
+    <t>39.4-41.4</t>
+  </si>
+  <si>
+    <t>70/60</t>
+  </si>
+  <si>
+    <t>2.7/4.7</t>
+  </si>
+  <si>
+    <t>2.6/4.5</t>
+  </si>
+  <si>
+    <t>1450/1545
+（副配重）</t>
+  </si>
+  <si>
+    <t>1450/1585/1626
+（副配重）</t>
+  </si>
+  <si>
+    <t>1610-1982
+（副配重影响）</t>
+  </si>
+  <si>
+    <t>1377-1709
+（副配重影响）</t>
   </si>
 </sst>
 </file>
@@ -713,7 +702,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -757,6 +746,24 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
@@ -781,23 +788,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1151,35 +1143,35 @@
         <v>11</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>128</v>
+        <v>96</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>129</v>
+        <v>97</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>130</v>
+        <v>98</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>131</v>
+        <v>99</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>132</v>
+        <v>100</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>133</v>
+        <v>101</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>134</v>
+        <v>102</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>135</v>
+        <v>103</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>136</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1189,35 +1181,35 @@
         <v>13</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>95</v>
+        <v>125</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>101</v>
+        <v>128</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>106</v>
+        <v>132</v>
+      </c>
+      <c r="G2" s="8">
+        <v>8891</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>109</v>
+        <v>137</v>
       </c>
       <c r="I2" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="J2" s="8" t="s">
-        <v>118</v>
+        <v>142</v>
+      </c>
+      <c r="J2" s="8">
+        <v>8630</v>
       </c>
       <c r="K2" s="8">
-        <v>5650</v>
+        <v>9537</v>
       </c>
       <c r="L2" s="8">
-        <v>5740</v>
+        <v>8800</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A3" s="16"/>
+      <c r="A3" s="22"/>
       <c r="B3" s="3" t="s">
         <v>14</v>
       </c>
@@ -1225,35 +1217,35 @@
         <v>15</v>
       </c>
       <c r="D3" s="3">
-        <v>1960</v>
+        <v>2300</v>
       </c>
       <c r="E3" s="8">
-        <v>1980</v>
+        <v>2300</v>
       </c>
       <c r="F3" s="8">
-        <v>2000</v>
+        <v>2200</v>
       </c>
       <c r="G3" s="8">
-        <v>1960</v>
+        <v>2200</v>
       </c>
       <c r="H3" s="8">
-        <v>1960</v>
+        <v>2200</v>
       </c>
       <c r="I3" s="8">
-        <v>1960</v>
+        <v>2300</v>
       </c>
       <c r="J3" s="8">
-        <v>2000</v>
+        <v>2300</v>
       </c>
       <c r="K3" s="8">
-        <v>2000</v>
+        <v>2250</v>
       </c>
       <c r="L3" s="8">
-        <v>1980</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A4" s="16"/>
+      <c r="A4" s="22"/>
       <c r="B4" s="3" t="s">
         <v>16</v>
       </c>
@@ -1261,35 +1253,35 @@
         <v>15</v>
       </c>
       <c r="D4" s="3">
-        <v>2555</v>
+        <v>2730</v>
       </c>
       <c r="E4" s="8">
+        <v>2660</v>
+      </c>
+      <c r="F4" s="8">
+        <v>2520</v>
+      </c>
+      <c r="G4" s="8">
+        <v>2540</v>
+      </c>
+      <c r="H4" s="8">
+        <v>2540</v>
+      </c>
+      <c r="I4" s="8">
+        <v>2715</v>
+      </c>
+      <c r="J4" s="8">
+        <v>2560</v>
+      </c>
+      <c r="K4" s="8">
+        <v>2657</v>
+      </c>
+      <c r="L4" s="8">
         <v>2550</v>
       </c>
-      <c r="F4" s="8">
-        <v>2530</v>
-      </c>
-      <c r="G4" s="8">
-        <v>2545</v>
-      </c>
-      <c r="H4" s="8">
-        <v>2550</v>
-      </c>
-      <c r="I4" s="8">
-        <v>2550</v>
-      </c>
-      <c r="J4" s="8">
-        <v>2540</v>
-      </c>
-      <c r="K4" s="8">
-        <v>2555</v>
-      </c>
-      <c r="L4" s="8">
-        <v>2575</v>
-      </c>
     </row>
     <row r="5" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A5" s="21"/>
+      <c r="A5" s="27"/>
       <c r="B5" s="4" t="s">
         <v>17</v>
       </c>
@@ -1297,35 +1289,35 @@
         <v>15</v>
       </c>
       <c r="D5" s="3">
-        <v>5340</v>
+        <v>6585</v>
       </c>
       <c r="E5" s="8">
-        <v>5305</v>
+        <v>6574</v>
       </c>
       <c r="F5" s="8">
-        <v>5470</v>
+        <v>6790</v>
       </c>
       <c r="G5" s="8">
-        <v>5368</v>
+        <v>6341</v>
       </c>
       <c r="H5" s="8">
-        <v>5435</v>
+        <v>6450</v>
       </c>
       <c r="I5" s="8">
-        <v>5520</v>
+        <v>6370</v>
       </c>
       <c r="J5" s="8">
-        <v>5198</v>
+        <v>6585</v>
       </c>
       <c r="K5" s="8">
-        <v>5510</v>
+        <v>6430</v>
       </c>
       <c r="L5" s="8">
-        <v>5445</v>
+        <v>7010</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="28" t="s">
         <v>1</v>
       </c>
       <c r="B6" s="5" t="s">
@@ -1335,35 +1327,35 @@
         <v>15</v>
       </c>
       <c r="D6" s="3">
-        <v>1560</v>
+        <v>1850</v>
       </c>
       <c r="E6" s="8">
-        <v>1580</v>
+        <v>1850</v>
       </c>
       <c r="F6" s="8">
-        <v>1600</v>
-      </c>
-      <c r="G6" s="8">
-        <v>1560</v>
+        <v>1750</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>32</v>
       </c>
       <c r="H6" s="8">
-        <v>1560</v>
+        <v>1750</v>
       </c>
       <c r="I6" s="8">
-        <v>1560</v>
+        <v>1850</v>
       </c>
       <c r="J6" s="8">
-        <v>1600</v>
+        <v>1850</v>
       </c>
       <c r="K6" s="8">
-        <v>1600</v>
+        <v>1800</v>
       </c>
       <c r="L6" s="8">
-        <v>1580</v>
+        <v>1750</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A7" s="16"/>
+      <c r="A7" s="22"/>
       <c r="B7" s="3" t="s">
         <v>19</v>
       </c>
@@ -1371,35 +1363,35 @@
         <v>15</v>
       </c>
       <c r="D7" s="3">
-        <v>1990</v>
+        <v>2272</v>
       </c>
       <c r="E7" s="8" t="s">
         <v>32</v>
       </c>
       <c r="F7" s="8">
-        <v>2000</v>
+        <v>2300</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>32</v>
       </c>
       <c r="H7" s="8">
-        <v>1990</v>
+        <v>2300</v>
       </c>
       <c r="I7" s="8">
-        <v>1990</v>
+        <v>2200</v>
       </c>
       <c r="J7" s="8">
-        <v>2000</v>
+        <v>2300</v>
       </c>
       <c r="K7" s="8">
-        <v>2000</v>
+        <v>2315</v>
       </c>
       <c r="L7" s="8">
-        <v>1990</v>
+        <v>2315</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A8" s="16"/>
+      <c r="A8" s="22"/>
       <c r="B8" s="3" t="s">
         <v>20</v>
       </c>
@@ -1407,35 +1399,35 @@
         <v>15</v>
       </c>
       <c r="D8" s="3">
-        <v>2490</v>
+        <v>2900</v>
       </c>
       <c r="E8" s="8">
-        <v>2580</v>
+        <v>2880</v>
       </c>
       <c r="F8" s="8">
-        <v>2500</v>
+        <v>2900</v>
       </c>
       <c r="G8" s="8" t="s">
         <v>32</v>
       </c>
       <c r="H8" s="8">
-        <v>2500</v>
+        <v>2900</v>
       </c>
       <c r="I8" s="8">
-        <v>2500</v>
+        <v>2830</v>
       </c>
       <c r="J8" s="8">
-        <v>2521</v>
+        <v>2885</v>
       </c>
       <c r="K8" s="8">
-        <v>2515</v>
+        <v>2952</v>
       </c>
       <c r="L8" s="8">
-        <v>2497</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A9" s="21"/>
+      <c r="A9" s="27"/>
       <c r="B9" s="4" t="s">
         <v>21</v>
       </c>
@@ -1443,35 +1435,35 @@
         <v>15</v>
       </c>
       <c r="D9" s="3">
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="E9" s="8">
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="F9" s="8">
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="G9" s="8">
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="H9" s="8">
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="I9" s="8">
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="J9" s="8">
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="K9" s="8">
-        <v>400</v>
+        <v>450</v>
       </c>
       <c r="L9" s="8">
-        <v>400</v>
+        <v>450</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="28" t="s">
         <v>22</v>
       </c>
       <c r="B10" s="5" t="s">
@@ -1481,35 +1473,35 @@
         <v>15</v>
       </c>
       <c r="D10" s="3">
-        <v>5650</v>
+        <v>6850</v>
       </c>
       <c r="E10" s="8">
-        <v>5215</v>
+        <v>6736</v>
       </c>
       <c r="F10" s="8">
-        <v>5750</v>
+        <v>7190</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>32</v>
       </c>
       <c r="H10" s="8">
-        <v>5635</v>
+        <v>7300</v>
       </c>
       <c r="I10" s="8">
-        <v>5785</v>
+        <v>6790</v>
       </c>
       <c r="J10" s="8">
-        <v>5369</v>
+        <v>6980</v>
       </c>
       <c r="K10" s="8">
-        <v>5740</v>
+        <v>6690</v>
       </c>
       <c r="L10" s="8">
-        <v>5585</v>
+        <v>7315</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A11" s="16"/>
+      <c r="A11" s="22"/>
       <c r="B11" s="3" t="s">
         <v>24</v>
       </c>
@@ -1517,35 +1509,35 @@
         <v>15</v>
       </c>
       <c r="D11" s="3">
-        <v>4010</v>
+        <v>4988</v>
       </c>
       <c r="E11" s="8">
-        <v>3700</v>
+        <v>4760</v>
       </c>
       <c r="F11" s="8">
-        <v>4070</v>
+        <v>5120</v>
       </c>
       <c r="G11" s="8">
-        <v>3975</v>
+        <v>5029</v>
       </c>
       <c r="H11" s="8">
-        <v>4000</v>
+        <v>5250</v>
       </c>
       <c r="I11" s="8">
-        <v>4155</v>
+        <v>4960</v>
       </c>
       <c r="J11" s="8">
-        <v>3787</v>
+        <v>4950</v>
       </c>
       <c r="K11" s="8">
-        <v>4035</v>
+        <v>4705</v>
       </c>
       <c r="L11" s="8">
-        <v>3835</v>
+        <v>5430</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A12" s="16"/>
+      <c r="A12" s="22"/>
       <c r="B12" s="3" t="s">
         <v>25</v>
       </c>
@@ -1553,35 +1545,35 @@
         <v>15</v>
       </c>
       <c r="D12" s="3">
-        <v>3640</v>
+        <v>3993</v>
       </c>
       <c r="E12" s="8">
-        <v>3420</v>
+        <v>4108</v>
       </c>
       <c r="F12" s="8">
-        <v>3530</v>
+        <v>4530</v>
       </c>
       <c r="G12" s="8">
-        <v>3478</v>
+        <v>4622</v>
       </c>
       <c r="H12" s="8">
-        <v>3630</v>
+        <v>4600</v>
       </c>
       <c r="I12" s="8">
-        <v>3875</v>
+        <v>4130</v>
       </c>
       <c r="J12" s="8">
-        <v>3716</v>
+        <v>4290</v>
       </c>
       <c r="K12" s="8">
-        <v>3750</v>
+        <v>4110</v>
       </c>
       <c r="L12" s="8">
-        <v>3630</v>
+        <v>4534</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A13" s="16"/>
+      <c r="A13" s="22"/>
       <c r="B13" s="3" t="s">
         <v>26</v>
       </c>
@@ -1589,107 +1581,105 @@
         <v>15</v>
       </c>
       <c r="D13" s="3">
-        <v>6110</v>
+        <v>7145</v>
       </c>
       <c r="E13" s="8">
-        <v>5755</v>
+        <v>7141</v>
       </c>
       <c r="F13" s="8">
-        <v>5960</v>
-      </c>
-      <c r="G13" s="8" t="s">
-        <v>32</v>
+        <v>7560</v>
+      </c>
+      <c r="G13" s="8">
+        <v>7176</v>
       </c>
       <c r="H13" s="8">
-        <v>6105</v>
+        <v>7330</v>
       </c>
       <c r="I13" s="8">
-        <v>6260</v>
+        <v>6970</v>
       </c>
       <c r="J13" s="8">
-        <v>5879</v>
+        <v>7090</v>
       </c>
       <c r="K13" s="8">
-        <v>6230</v>
-      </c>
-      <c r="L13" s="8">
-        <v>6080</v>
+        <v>7015</v>
+      </c>
+      <c r="L13" s="3" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A14" s="16"/>
+      <c r="A14" s="22"/>
       <c r="B14" s="3" t="s">
         <v>27</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D14" s="3">
-        <v>5960</v>
+      <c r="D14" s="3" t="s">
+        <v>32</v>
       </c>
       <c r="E14" s="8">
-        <v>5590</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="G14" s="8">
-        <v>5889</v>
+        <v>6949</v>
+      </c>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8" t="s">
+        <v>32</v>
       </c>
       <c r="H14" s="8">
-        <v>5965</v>
+        <v>7170</v>
       </c>
       <c r="I14" s="8">
-        <v>6125</v>
+        <v>6800</v>
       </c>
       <c r="J14" s="8">
-        <v>5748</v>
+        <v>6940</v>
       </c>
       <c r="K14" s="8">
-        <v>6100</v>
+        <v>6850</v>
       </c>
       <c r="L14" s="8">
-        <v>5950</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="28.15" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A15" s="21"/>
+        <v>7115</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="55.9" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A15" s="27"/>
       <c r="B15" s="4" t="s">
         <v>28</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D15" s="3">
-        <v>1040</v>
-      </c>
-      <c r="E15" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="F15" s="12" t="s">
-        <v>122</v>
+      <c r="D15" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="F15" s="10">
+        <v>1590</v>
       </c>
       <c r="G15" s="7" t="s">
         <v>32</v>
       </c>
       <c r="H15" s="7">
-        <v>1065</v>
-      </c>
-      <c r="I15" s="7">
-        <v>1270</v>
-      </c>
-      <c r="J15" s="10" t="s">
-        <v>123</v>
+        <v>1460</v>
+      </c>
+      <c r="I15" s="10">
+        <v>1290</v>
+      </c>
+      <c r="J15" s="10">
+        <v>1600</v>
       </c>
       <c r="K15" s="10">
-        <v>1175</v>
-      </c>
-      <c r="L15" s="10">
-        <v>1050</v>
+        <v>1465</v>
+      </c>
+      <c r="L15" s="7">
+        <v>1480</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="28" t="s">
         <v>2</v>
       </c>
       <c r="B16" s="5" t="s">
@@ -1699,35 +1689,33 @@
         <v>30</v>
       </c>
       <c r="D16" s="3">
-        <v>30.7</v>
+        <v>54.6</v>
       </c>
       <c r="E16" s="12">
-        <v>36.1</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="G16" s="7">
-        <v>36.5</v>
+        <v>55.4</v>
+      </c>
+      <c r="F16" s="12"/>
+      <c r="G16" s="7" t="s">
+        <v>32</v>
       </c>
       <c r="H16" s="7">
-        <v>35.5</v>
-      </c>
-      <c r="I16" s="7">
-        <v>35.5</v>
-      </c>
-      <c r="J16" s="7">
-        <v>31.2</v>
+        <v>49.7</v>
+      </c>
+      <c r="I16" s="17">
+        <v>42.4</v>
+      </c>
+      <c r="J16" s="8">
+        <v>49.9</v>
       </c>
       <c r="K16" s="8">
-        <v>35.5</v>
+        <v>48.5</v>
       </c>
       <c r="L16" s="8">
-        <v>36.4</v>
+        <v>53.7</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A17" s="21"/>
+      <c r="A17" s="27"/>
       <c r="B17" s="4" t="s">
         <v>31</v>
       </c>
@@ -1738,32 +1726,32 @@
         <v>32</v>
       </c>
       <c r="E17" s="8">
-        <v>33.6</v>
+        <v>51.8</v>
       </c>
       <c r="F17" s="8">
-        <v>26.8</v>
-      </c>
-      <c r="G17" s="7" t="s">
-        <v>32</v>
+        <v>50.4</v>
+      </c>
+      <c r="G17" s="7">
+        <v>48.7</v>
       </c>
       <c r="H17" s="8">
-        <v>34.6</v>
-      </c>
-      <c r="I17" s="8">
-        <v>34.6</v>
-      </c>
-      <c r="J17" s="7" t="s">
-        <v>32</v>
+        <v>46.5</v>
+      </c>
+      <c r="I17" s="17">
+        <v>41</v>
+      </c>
+      <c r="J17" s="8">
+        <v>48.5</v>
       </c>
       <c r="K17" s="8">
-        <v>33.6</v>
+        <v>47.1</v>
       </c>
       <c r="L17" s="8">
-        <v>35.1</v>
+        <v>49.5</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="28" t="s">
         <v>33</v>
       </c>
       <c r="B18" s="5" t="s">
@@ -1773,13 +1761,13 @@
         <v>15</v>
       </c>
       <c r="D18" s="3">
-        <v>1570</v>
+        <v>1823</v>
       </c>
       <c r="E18" s="8">
-        <v>1351</v>
+        <v>1820</v>
       </c>
       <c r="F18" s="8">
-        <v>1380</v>
+        <v>2120</v>
       </c>
       <c r="G18" s="7" t="s">
         <v>32</v>
@@ -1787,21 +1775,21 @@
       <c r="H18" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="I18" s="7" t="s">
-        <v>32</v>
+      <c r="I18" s="8">
+        <v>1700</v>
       </c>
       <c r="J18" s="8">
-        <v>1400</v>
+        <v>1750</v>
       </c>
       <c r="K18" s="8">
-        <v>1650</v>
+        <v>1700</v>
       </c>
       <c r="L18" s="8">
-        <v>1600</v>
+        <v>2051</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A19" s="16"/>
+      <c r="A19" s="22"/>
       <c r="B19" s="3" t="s">
         <v>35</v>
       </c>
@@ -1809,13 +1797,13 @@
         <v>15</v>
       </c>
       <c r="D19" s="3">
-        <v>2850</v>
+        <v>3400</v>
       </c>
       <c r="E19" s="8">
-        <v>2716</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>32</v>
+        <v>3400</v>
+      </c>
+      <c r="F19" s="8">
+        <v>3670</v>
       </c>
       <c r="G19" s="7" t="s">
         <v>32</v>
@@ -1823,36 +1811,34 @@
       <c r="H19" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="I19" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="J19" s="7">
-        <v>2750</v>
+      <c r="I19" s="7">
+        <v>3550</v>
+      </c>
+      <c r="J19" s="8">
+        <v>3550</v>
       </c>
       <c r="K19" s="8">
-        <v>2800</v>
+        <v>3380</v>
       </c>
       <c r="L19" s="8">
-        <v>2700</v>
+        <v>3520</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A20" s="21"/>
+      <c r="A20" s="27"/>
       <c r="B20" s="4" t="s">
         <v>36</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D20" s="7">
-        <v>1900</v>
-      </c>
-      <c r="E20" s="8">
-        <v>1601</v>
-      </c>
-      <c r="F20" s="8">
-        <v>1690</v>
-      </c>
+      <c r="D20" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E20" s="29">
+        <v>2358</v>
+      </c>
+      <c r="F20" s="7"/>
       <c r="G20" s="7" t="s">
         <v>32</v>
       </c>
@@ -1862,18 +1848,18 @@
       <c r="I20" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="J20" s="8">
-        <v>1800</v>
-      </c>
-      <c r="K20" s="8">
-        <v>1400</v>
-      </c>
-      <c r="L20" s="8">
-        <v>1900</v>
+      <c r="J20" s="7">
+        <v>2100</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="L20" s="7" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A21" s="22" t="s">
+      <c r="A21" s="28" t="s">
         <v>3</v>
       </c>
       <c r="B21" s="5" t="s">
@@ -1885,33 +1871,33 @@
       <c r="D21" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="E21" s="3" t="s">
         <v>38</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>124</v>
+        <v>89</v>
       </c>
       <c r="G21" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="H21" s="7" t="s">
-        <v>89</v>
+      <c r="H21" s="3" t="s">
+        <v>38</v>
       </c>
       <c r="I21" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="J21" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="K21" s="7" t="s">
+      <c r="J21" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="L21" s="13" t="s">
+      <c r="K21" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="L21" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A22" s="16"/>
+      <c r="A22" s="22"/>
       <c r="B22" s="3" t="s">
         <v>39</v>
       </c>
@@ -1919,35 +1905,35 @@
         <v>40</v>
       </c>
       <c r="D22" s="3">
-        <v>158.4</v>
+        <v>219</v>
       </c>
       <c r="E22" s="8">
+        <v>167</v>
+      </c>
+      <c r="F22" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="F22" s="8">
-        <v>120</v>
-      </c>
       <c r="G22" s="7" t="s">
         <v>32</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>110</v>
+        <v>138</v>
       </c>
       <c r="I22" s="8" t="s">
-        <v>114</v>
+        <v>143</v>
       </c>
       <c r="J22" s="8">
-        <v>120</v>
-      </c>
-      <c r="K22" s="8">
-        <v>138</v>
-      </c>
-      <c r="L22" s="14">
-        <v>139</v>
+        <v>144</v>
+      </c>
+      <c r="K22" s="14">
+        <v>149</v>
+      </c>
+      <c r="L22" s="8">
+        <v>193</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A23" s="16"/>
+      <c r="A23" s="22"/>
       <c r="B23" s="3" t="s">
         <v>41</v>
       </c>
@@ -1955,13 +1941,13 @@
         <v>42</v>
       </c>
       <c r="D23" s="3">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E23" s="8">
-        <v>26.5</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>32</v>
+        <v>28.5</v>
+      </c>
+      <c r="F23" s="8">
+        <v>28</v>
       </c>
       <c r="G23" s="7" t="s">
         <v>32</v>
@@ -1969,21 +1955,21 @@
       <c r="H23" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="I23" s="7" t="s">
-        <v>32</v>
+      <c r="I23" s="8">
+        <v>29.4</v>
       </c>
       <c r="J23" s="8">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="K23" s="8">
-        <v>25.4</v>
-      </c>
-      <c r="L23" s="1">
-        <v>30.1</v>
+        <v>29.5</v>
+      </c>
+      <c r="L23" s="8">
+        <v>26.3</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A24" s="16"/>
+      <c r="A24" s="22"/>
       <c r="B24" s="3" t="s">
         <v>43</v>
       </c>
@@ -1991,13 +1977,13 @@
         <v>42</v>
       </c>
       <c r="D24" s="3">
-        <v>28.4</v>
+        <v>30</v>
       </c>
       <c r="E24" s="8">
-        <v>26.5</v>
-      </c>
-      <c r="F24" s="7" t="s">
-        <v>32</v>
+        <v>28.5</v>
+      </c>
+      <c r="F24" s="8">
+        <v>31.6</v>
       </c>
       <c r="G24" s="7" t="s">
         <v>32</v>
@@ -2005,21 +1991,21 @@
       <c r="H24" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="I24" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="J24" s="7" t="s">
-        <v>32</v>
+      <c r="I24" s="7">
+        <v>29.4</v>
+      </c>
+      <c r="J24" s="8">
+        <v>28</v>
       </c>
       <c r="K24" s="8">
-        <v>28.5</v>
-      </c>
-      <c r="L24" s="13" t="s">
-        <v>32</v>
+        <v>29.5</v>
+      </c>
+      <c r="L24" s="8">
+        <v>26.3</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A25" s="16"/>
+      <c r="A25" s="22"/>
       <c r="B25" s="3" t="s">
         <v>44</v>
       </c>
@@ -2027,13 +2013,13 @@
         <v>42</v>
       </c>
       <c r="D25" s="3">
-        <v>23</v>
+        <v>23.5</v>
       </c>
       <c r="E25" s="8">
-        <v>20</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>32</v>
+        <v>25</v>
+      </c>
+      <c r="F25" s="8">
+        <v>26.1</v>
       </c>
       <c r="G25" s="7" t="s">
         <v>32</v>
@@ -2041,165 +2027,157 @@
       <c r="H25" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="I25" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="J25" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="K25" s="8">
-        <v>35</v>
-      </c>
-      <c r="L25" s="13">
+      <c r="I25" s="7">
+        <v>24.5</v>
+      </c>
+      <c r="J25" s="8">
+        <v>25</v>
+      </c>
+      <c r="K25" s="13">
         <v>21.6</v>
       </c>
+      <c r="L25" s="7" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A26" s="16"/>
+      <c r="A26" s="22"/>
       <c r="B26" s="3" t="s">
         <v>45</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D26" s="3">
-        <v>110</v>
+      <c r="D26" s="7" t="s">
+        <v>32</v>
       </c>
       <c r="E26" s="8">
-        <v>80</v>
-      </c>
-      <c r="F26" s="8">
-        <v>87.4</v>
-      </c>
+        <v>131</v>
+      </c>
+      <c r="F26" s="8"/>
       <c r="G26" s="8">
-        <v>75.7</v>
+        <v>95</v>
       </c>
       <c r="H26" s="8">
-        <v>75</v>
-      </c>
-      <c r="I26" s="8">
-        <v>76</v>
-      </c>
-      <c r="J26" s="8">
-        <v>75</v>
-      </c>
-      <c r="K26" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="L26" s="13" t="s">
-        <v>32</v>
+        <v>100</v>
+      </c>
+      <c r="I26" s="7">
+        <v>118</v>
+      </c>
+      <c r="J26" s="7">
+        <v>100</v>
+      </c>
+      <c r="K26" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="L26" s="8">
+        <v>100</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A27" s="16"/>
+      <c r="A27" s="22"/>
       <c r="B27" s="3" t="s">
         <v>46</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D27" s="3">
-        <v>21</v>
+      <c r="D27" s="7" t="s">
+        <v>32</v>
       </c>
       <c r="E27" s="12">
-        <v>26.5</v>
-      </c>
-      <c r="F27" s="7" t="s">
-        <v>32</v>
-      </c>
+        <v>28.5</v>
+      </c>
+      <c r="F27" s="12"/>
       <c r="G27" s="8">
         <v>21</v>
       </c>
       <c r="H27" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="I27" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="J27" s="8">
-        <v>22</v>
-      </c>
-      <c r="K27" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="L27" s="13" t="s">
-        <v>32</v>
+      <c r="I27" s="7">
+        <v>21.6</v>
+      </c>
+      <c r="J27" s="7">
+        <v>18</v>
+      </c>
+      <c r="K27" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="L27" s="8">
+        <v>25</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A28" s="16"/>
+      <c r="A28" s="22"/>
       <c r="B28" s="3" t="s">
         <v>48</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D28" s="3">
-        <v>75</v>
+      <c r="D28" s="7" t="s">
+        <v>32</v>
       </c>
       <c r="E28" s="8">
-        <v>28</v>
-      </c>
-      <c r="F28" s="7" t="s">
-        <v>32</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="F28" s="8"/>
       <c r="G28" s="7" t="s">
         <v>32</v>
       </c>
       <c r="H28" s="7">
-        <v>37</v>
+        <v>55.8</v>
       </c>
       <c r="I28" s="7">
-        <v>38</v>
-      </c>
-      <c r="J28" s="8">
-        <v>40</v>
-      </c>
-      <c r="K28" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="L28" s="13" t="s">
-        <v>32</v>
+        <v>68</v>
+      </c>
+      <c r="J28" s="7">
+        <v>57</v>
+      </c>
+      <c r="K28" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="L28" s="7">
+        <v>70</v>
       </c>
     </row>
     <row r="29" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A29" s="21"/>
+      <c r="A29" s="27"/>
       <c r="B29" s="4" t="s">
         <v>49</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D29" s="3">
-        <v>17</v>
+      <c r="D29" s="7" t="s">
+        <v>32</v>
       </c>
       <c r="E29" s="8">
-        <v>26.5</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>32</v>
-      </c>
+        <v>28.5</v>
+      </c>
+      <c r="F29" s="8"/>
       <c r="G29" s="7" t="s">
         <v>32</v>
       </c>
       <c r="H29" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="I29" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="J29" s="8">
-        <v>22</v>
-      </c>
-      <c r="K29" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="L29" s="13" t="s">
-        <v>32</v>
+      <c r="I29" s="7">
+        <v>29.4</v>
+      </c>
+      <c r="J29" s="7">
+        <v>28</v>
+      </c>
+      <c r="K29" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="L29" s="7">
+        <v>25</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A30" s="18" t="s">
+      <c r="A30" s="24" t="s">
         <v>4</v>
       </c>
       <c r="B30" s="5" t="s">
@@ -2209,35 +2187,35 @@
         <v>51</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>96</v>
+        <v>126</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>98</v>
+        <v>129</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>103</v>
+        <v>134</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>111</v>
+        <v>139</v>
       </c>
       <c r="I30" s="8" t="s">
-        <v>115</v>
+        <v>144</v>
       </c>
       <c r="J30" s="8" t="s">
-        <v>119</v>
+        <v>92</v>
       </c>
       <c r="K30" s="8" t="s">
-        <v>90</v>
+        <v>147</v>
       </c>
       <c r="L30" s="8" t="s">
-        <v>92</v>
+        <v>148</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A31" s="19"/>
+      <c r="A31" s="25"/>
       <c r="B31" s="3" t="s">
         <v>52</v>
       </c>
@@ -2245,35 +2223,35 @@
         <v>53</v>
       </c>
       <c r="D31" s="3">
-        <v>52.8</v>
+        <v>64</v>
       </c>
       <c r="E31" s="8">
-        <v>50.5</v>
-      </c>
-      <c r="F31" s="8" t="s">
-        <v>32</v>
+        <v>67.5</v>
+      </c>
+      <c r="F31" s="8">
+        <v>63.9</v>
       </c>
       <c r="G31" s="7" t="s">
         <v>32</v>
       </c>
       <c r="H31" s="8">
-        <v>45.1</v>
-      </c>
-      <c r="I31" s="8">
-        <v>64.400000000000006</v>
+        <v>67</v>
+      </c>
+      <c r="I31" s="16">
+        <v>65</v>
       </c>
       <c r="J31" s="8">
-        <v>38.299999999999997</v>
+        <v>62.8</v>
       </c>
       <c r="K31" s="8">
-        <v>55.5</v>
+        <v>64.7</v>
       </c>
       <c r="L31" s="8">
-        <v>44.9</v>
+        <v>70</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A32" s="19"/>
+      <c r="A32" s="25"/>
       <c r="B32" s="3" t="s">
         <v>54</v>
       </c>
@@ -2281,35 +2259,35 @@
         <v>55</v>
       </c>
       <c r="D32" s="3">
-        <v>32</v>
+        <v>42.8</v>
       </c>
       <c r="E32" s="8" t="s">
-        <v>99</v>
+        <v>130</v>
       </c>
       <c r="F32" s="8" t="s">
-        <v>104</v>
+        <v>135</v>
       </c>
       <c r="G32" s="8">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="H32" s="8" t="s">
-        <v>112</v>
+        <v>140</v>
       </c>
       <c r="I32" s="8" t="s">
-        <v>116</v>
+        <v>145</v>
       </c>
       <c r="J32" s="8">
-        <v>28.4</v>
+        <v>37.5</v>
       </c>
       <c r="K32" s="8">
-        <v>32.1</v>
+        <v>41.4</v>
       </c>
       <c r="L32" s="8">
-        <v>32.4</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="33" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A33" s="20"/>
+      <c r="A33" s="26"/>
       <c r="B33" s="4" t="s">
         <v>56</v>
       </c>
@@ -2322,20 +2300,18 @@
       <c r="E33" s="8">
         <v>30</v>
       </c>
-      <c r="F33" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="G33" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="H33" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="I33" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="J33" s="7">
-        <v>20</v>
+      <c r="F33" s="8"/>
+      <c r="G33" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="H33" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="I33" s="7">
+        <v>35</v>
+      </c>
+      <c r="J33" s="8">
+        <v>35</v>
       </c>
       <c r="K33" s="8">
         <v>35</v>
@@ -2345,7 +2321,7 @@
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A34" s="18" t="s">
+      <c r="A34" s="24" t="s">
         <v>5</v>
       </c>
       <c r="B34" s="5" t="s">
@@ -2355,35 +2331,35 @@
         <v>59</v>
       </c>
       <c r="D34" s="3">
+        <v>12</v>
+      </c>
+      <c r="E34" s="8">
+        <v>10.6</v>
+      </c>
+      <c r="F34" s="8">
+        <v>10.1</v>
+      </c>
+      <c r="G34" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="H34" s="8">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="I34" s="16">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="J34" s="8">
+        <v>9</v>
+      </c>
+      <c r="K34" s="8">
         <v>9.5</v>
       </c>
-      <c r="E34" s="8">
-        <v>9</v>
-      </c>
-      <c r="F34" s="8">
-        <v>9</v>
-      </c>
-      <c r="G34" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="H34" s="8">
-        <v>9.1999999999999993</v>
-      </c>
-      <c r="I34" s="8">
-        <v>9.1999999999999993</v>
-      </c>
-      <c r="J34" s="8">
-        <v>8.5</v>
-      </c>
-      <c r="K34" s="8">
-        <v>10.1</v>
-      </c>
       <c r="L34" s="8">
-        <v>9.8000000000000007</v>
+        <v>11</v>
       </c>
     </row>
     <row r="35" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A35" s="20"/>
+      <c r="A35" s="26"/>
       <c r="B35" s="4" t="s">
         <v>60</v>
       </c>
@@ -2391,35 +2367,35 @@
         <v>57</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>97</v>
+        <v>127</v>
       </c>
       <c r="E35" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="F35" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="G35" s="7" t="s">
-        <v>108</v>
+        <v>131</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="G35" s="8" t="s">
+        <v>32</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>97</v>
+        <v>141</v>
       </c>
       <c r="I35" s="7" t="s">
-        <v>117</v>
-      </c>
-      <c r="J35" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="K35" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="J35" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="K35" s="8" t="s">
         <v>32</v>
       </c>
       <c r="L35" s="7" t="s">
-        <v>120</v>
+        <v>32</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A36" s="18" t="s">
+      <c r="A36" s="24" t="s">
         <v>6</v>
       </c>
       <c r="B36" s="5" t="s">
@@ -2429,35 +2405,35 @@
         <v>53</v>
       </c>
       <c r="D36" s="3">
-        <v>44.5</v>
+        <v>64</v>
       </c>
       <c r="E36" s="8">
-        <v>49.2</v>
+        <v>62</v>
       </c>
       <c r="F36" s="8">
-        <v>36.799999999999997</v>
+        <v>59</v>
       </c>
       <c r="G36" s="8">
-        <v>42.3</v>
+        <v>67.3</v>
       </c>
       <c r="H36" s="8">
-        <v>45.2</v>
+        <v>65.2</v>
       </c>
       <c r="I36" s="8">
-        <v>45.2</v>
+        <v>57.2</v>
       </c>
       <c r="J36" s="8">
-        <v>36.200000000000003</v>
+        <v>68.3</v>
       </c>
       <c r="K36" s="8">
-        <v>37</v>
+        <v>65.7</v>
       </c>
       <c r="L36" s="8">
-        <v>43.4</v>
+        <v>72.7</v>
       </c>
     </row>
     <row r="37" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A37" s="20"/>
+      <c r="A37" s="26"/>
       <c r="B37" s="4" t="s">
         <v>62</v>
       </c>
@@ -2465,39 +2441,39 @@
         <v>53</v>
       </c>
       <c r="D37" s="3">
-        <v>24.3</v>
+        <v>41</v>
       </c>
       <c r="E37" s="8">
-        <v>28.6</v>
+        <v>42.3</v>
       </c>
       <c r="F37" s="8">
-        <v>24</v>
+        <v>35.299999999999997</v>
       </c>
       <c r="G37" s="8">
-        <v>31.1</v>
+        <v>38.299999999999997</v>
       </c>
       <c r="H37" s="8">
-        <v>26.1</v>
+        <v>38</v>
       </c>
       <c r="I37" s="8">
-        <v>24.3</v>
+        <v>39.799999999999997</v>
       </c>
       <c r="J37" s="8">
-        <v>25.9</v>
+        <v>45.9</v>
       </c>
       <c r="K37" s="8">
-        <v>23</v>
+        <v>43.7</v>
       </c>
       <c r="L37" s="8">
-        <v>27.4</v>
+        <v>40.5</v>
       </c>
     </row>
     <row r="38" spans="1:12" ht="27.75" x14ac:dyDescent="0.45">
-      <c r="A38" s="18" t="s">
+      <c r="A38" s="24" t="s">
         <v>7</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>137</v>
+        <v>105</v>
       </c>
       <c r="C38" s="5" t="s">
         <v>13</v>
@@ -2506,13 +2482,13 @@
         <v>32</v>
       </c>
       <c r="E38" s="7">
-        <v>2587</v>
+        <v>3533</v>
       </c>
       <c r="F38" s="7">
-        <v>2511</v>
-      </c>
-      <c r="G38" s="7">
-        <v>3060</v>
+        <v>3207</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>32</v>
       </c>
       <c r="H38" s="7" t="s">
         <v>32</v>
@@ -2521,32 +2497,30 @@
         <v>32</v>
       </c>
       <c r="J38" s="7">
-        <v>2383</v>
+        <v>2830</v>
       </c>
       <c r="K38" s="7">
-        <v>2400</v>
-      </c>
-      <c r="L38" s="7">
-        <v>2780</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" ht="27.75" x14ac:dyDescent="0.45">
-      <c r="A39" s="19"/>
+        <v>2890</v>
+      </c>
+      <c r="L38" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" ht="55.5" x14ac:dyDescent="0.45">
+      <c r="A39" s="25"/>
       <c r="B39" s="3" t="s">
-        <v>138</v>
+        <v>106</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D39" s="3">
-        <v>1760</v>
-      </c>
-      <c r="E39" s="10">
-        <v>1953</v>
-      </c>
-      <c r="F39" s="7" t="s">
-        <v>32</v>
-      </c>
+      <c r="D39" s="7">
+        <v>1480</v>
+      </c>
+      <c r="E39" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="F39" s="10"/>
       <c r="G39" s="7" t="s">
         <v>32</v>
       </c>
@@ -2556,35 +2530,35 @@
       <c r="I39" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="J39" s="7">
-        <v>1626</v>
-      </c>
-      <c r="K39" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="L39" s="7">
-        <v>1610</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A40" s="20"/>
+      <c r="J39" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="K39" s="7">
+        <v>1770</v>
+      </c>
+      <c r="L39" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" ht="55.9" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A40" s="26"/>
       <c r="B40" s="4" t="s">
-        <v>139</v>
+        <v>107</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D40" s="3">
-        <v>1030</v>
-      </c>
-      <c r="E40" s="10">
-        <v>1579</v>
+      <c r="D40" s="7">
+        <v>1165</v>
+      </c>
+      <c r="E40" s="10" t="s">
+        <v>152</v>
       </c>
       <c r="F40" s="10">
-        <v>1150</v>
-      </c>
-      <c r="G40" s="7">
-        <v>1057</v>
+        <v>1430</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>32</v>
       </c>
       <c r="H40" s="7" t="s">
         <v>32</v>
@@ -2592,14 +2566,14 @@
       <c r="I40" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="J40" s="7">
-        <v>1092</v>
+      <c r="J40" s="10">
+        <v>1710</v>
       </c>
       <c r="K40" s="10">
-        <v>1400</v>
-      </c>
-      <c r="L40" s="10">
-        <v>1430</v>
+        <v>1520</v>
+      </c>
+      <c r="L40" s="7" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -2632,35 +2606,35 @@
       <c r="A1" s="2"/>
       <c r="B1" s="2"/>
       <c r="C1" s="2" t="s">
-        <v>128</v>
+        <v>96</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>129</v>
+        <v>97</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>130</v>
+        <v>98</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>131</v>
+        <v>99</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>132</v>
+        <v>100</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>133</v>
+        <v>101</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>134</v>
+        <v>102</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>135</v>
+        <v>103</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>136</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="21" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="6" t="s">
@@ -2695,7 +2669,7 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A3" s="16"/>
+      <c r="A3" s="22"/>
       <c r="B3" s="3" t="s">
         <v>65</v>
       </c>
@@ -2728,9 +2702,9 @@
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A4" s="16"/>
-      <c r="B4" s="23" t="s">
-        <v>140</v>
+      <c r="A4" s="22"/>
+      <c r="B4" s="15" t="s">
+        <v>108</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>70</v>
@@ -2761,7 +2735,7 @@
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A5" s="16"/>
+      <c r="A5" s="22"/>
       <c r="B5" s="1" t="s">
         <v>66</v>
       </c>
@@ -2794,7 +2768,7 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="14.65" x14ac:dyDescent="0.45">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="22" t="s">
         <v>67</v>
       </c>
       <c r="B6" s="9" t="s">
@@ -2829,7 +2803,7 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A7" s="16"/>
+      <c r="A7" s="22"/>
       <c r="B7" s="3" t="s">
         <v>69</v>
       </c>
@@ -2862,7 +2836,7 @@
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A8" s="16"/>
+      <c r="A8" s="22"/>
       <c r="B8" s="3" t="s">
         <v>71</v>
       </c>
@@ -2895,7 +2869,7 @@
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A9" s="16"/>
+      <c r="A9" s="22"/>
       <c r="B9" s="3" t="s">
         <v>72</v>
       </c>
@@ -2928,7 +2902,7 @@
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A10" s="16"/>
+      <c r="A10" s="22"/>
       <c r="B10" s="3" t="s">
         <v>73</v>
       </c>
@@ -2961,14 +2935,14 @@
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A11" s="16"/>
+      <c r="A11" s="22"/>
       <c r="B11" s="3" t="s">
-        <v>141</v>
+        <v>109</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="27" t="s">
+      <c r="D11" s="16" t="s">
         <v>70</v>
       </c>
       <c r="E11" s="7" t="s">
@@ -2994,7 +2968,7 @@
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A12" s="16"/>
+      <c r="A12" s="22"/>
       <c r="B12" s="3" t="s">
         <v>74</v>
       </c>
@@ -3027,7 +3001,7 @@
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A13" s="16"/>
+      <c r="A13" s="22"/>
       <c r="B13" s="3" t="s">
         <v>75</v>
       </c>
@@ -3044,7 +3018,7 @@
         <v>70</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="H13" s="7" t="s">
         <v>32</v>
@@ -3060,7 +3034,7 @@
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="22" t="s">
         <v>9</v>
       </c>
       <c r="B14" s="3" t="s">
@@ -3095,7 +3069,7 @@
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A15" s="16"/>
+      <c r="A15" s="22"/>
       <c r="B15" s="3" t="s">
         <v>77</v>
       </c>
@@ -3128,7 +3102,7 @@
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A16" s="16"/>
+      <c r="A16" s="22"/>
       <c r="B16" s="3" t="s">
         <v>78</v>
       </c>
@@ -3161,7 +3135,7 @@
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A17" s="16"/>
+      <c r="A17" s="22"/>
       <c r="B17" s="3" t="s">
         <v>79</v>
       </c>
@@ -3194,7 +3168,7 @@
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A18" s="16"/>
+      <c r="A18" s="22"/>
       <c r="B18" s="3" t="s">
         <v>80</v>
       </c>
@@ -3227,11 +3201,11 @@
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A19" s="17" t="s">
+      <c r="A19" s="23" t="s">
         <v>81</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>126</v>
+        <v>94</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>32</v>
@@ -3262,9 +3236,9 @@
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A20" s="17"/>
+      <c r="A20" s="23"/>
       <c r="B20" s="3" t="s">
-        <v>127</v>
+        <v>95</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>64</v>
@@ -3295,7 +3269,7 @@
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A21" s="17"/>
+      <c r="A21" s="23"/>
       <c r="B21" s="3" t="s">
         <v>82</v>
       </c>
@@ -3328,9 +3302,9 @@
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A22" s="17"/>
+      <c r="A22" s="23"/>
       <c r="B22" s="3" t="s">
-        <v>142</v>
+        <v>110</v>
       </c>
       <c r="C22" s="7" t="s">
         <v>32</v>
@@ -3361,7 +3335,7 @@
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A23" s="17"/>
+      <c r="A23" s="23"/>
       <c r="B23" s="3" t="s">
         <v>83</v>
       </c>
@@ -3394,15 +3368,15 @@
       </c>
     </row>
     <row r="24" spans="1:11" ht="27.75" x14ac:dyDescent="0.45">
-      <c r="A24" s="17"/>
+      <c r="A24" s="23"/>
       <c r="B24" s="3" t="s">
-        <v>143</v>
+        <v>111</v>
       </c>
       <c r="C24" s="7" t="s">
         <v>32</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>149</v>
+        <v>117</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>32</v>
@@ -3427,9 +3401,9 @@
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A25" s="17"/>
+      <c r="A25" s="23"/>
       <c r="B25" s="3" t="s">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>32</v>
@@ -3460,7 +3434,7 @@
       </c>
     </row>
     <row r="26" spans="1:11" ht="41.65" x14ac:dyDescent="0.45">
-      <c r="A26" s="17"/>
+      <c r="A26" s="23"/>
       <c r="B26" s="9" t="s">
         <v>84</v>
       </c>
@@ -3468,13 +3442,13 @@
         <v>32</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>148</v>
+        <v>116</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>32</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="G26" s="7" t="s">
         <v>32</v>
@@ -3493,11 +3467,11 @@
       </c>
     </row>
     <row r="27" spans="1:11" ht="27.75" x14ac:dyDescent="0.45">
-      <c r="A27" s="24" t="s">
+      <c r="A27" s="18" t="s">
         <v>10</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>145</v>
+        <v>113</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>32</v>
@@ -3518,7 +3492,7 @@
         <v>32</v>
       </c>
       <c r="I27" s="10" t="s">
-        <v>154</v>
+        <v>122</v>
       </c>
       <c r="J27" s="7" t="s">
         <v>32</v>
@@ -3528,7 +3502,7 @@
       </c>
     </row>
     <row r="28" spans="1:11" ht="27.75" x14ac:dyDescent="0.45">
-      <c r="A28" s="25"/>
+      <c r="A28" s="19"/>
       <c r="B28" s="3" t="s">
         <v>85</v>
       </c>
@@ -3536,7 +3510,7 @@
         <v>32</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>152</v>
+        <v>120</v>
       </c>
       <c r="E28" s="10" t="s">
         <v>64</v>
@@ -3548,20 +3522,20 @@
         <v>32</v>
       </c>
       <c r="H28" s="10" t="s">
-        <v>153</v>
+        <v>121</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>153</v>
+        <v>121</v>
       </c>
       <c r="J28" s="10" t="s">
-        <v>155</v>
+        <v>123</v>
       </c>
       <c r="K28" s="7" t="s">
-        <v>156</v>
+        <v>124</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A29" s="25"/>
+      <c r="A29" s="19"/>
       <c r="B29" s="3" t="s">
         <v>86</v>
       </c>
@@ -3594,14 +3568,14 @@
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A30" s="25"/>
+      <c r="A30" s="19"/>
       <c r="B30" s="3" t="s">
         <v>87</v>
       </c>
       <c r="C30" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="D30" s="28" t="s">
+      <c r="D30" s="17" t="s">
         <v>70</v>
       </c>
       <c r="E30" s="7" t="s">
@@ -3627,9 +3601,9 @@
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A31" s="25"/>
+      <c r="A31" s="19"/>
       <c r="B31" s="3" t="s">
-        <v>146</v>
+        <v>114</v>
       </c>
       <c r="C31" s="8" t="s">
         <v>70</v>
@@ -3660,9 +3634,9 @@
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A32" s="25"/>
+      <c r="A32" s="19"/>
       <c r="B32" s="3" t="s">
-        <v>147</v>
+        <v>115</v>
       </c>
       <c r="C32" s="7" t="s">
         <v>32</v>
@@ -3689,15 +3663,15 @@
       <c r="K32" s="10"/>
     </row>
     <row r="33" spans="1:11" ht="27.75" x14ac:dyDescent="0.45">
-      <c r="A33" s="26"/>
+      <c r="A33" s="20"/>
       <c r="B33" s="3" t="s">
         <v>88</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>150</v>
+        <v>118</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>151</v>
+        <v>119</v>
       </c>
       <c r="E33" s="10" t="s">
         <v>70</v>

</xml_diff>